<commit_message>
adjusting to logic in quality check
Moving cycle time logic into quality check - leads to warm up period of 2500
</commit_message>
<xml_diff>
--- a/baseline_cycle_times_1.xlsx
+++ b/baseline_cycle_times_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7b32c6e2a84854a2/Desktop/Edinburgh/University/Simulation/Simulation-Project-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_CBAE28510E3E71D7E7CB3A41CD3976629309777F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3BB34AB-549B-49F2-91A9-9486C9112693}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_CBAE28510E3E71D7E7CB3A41CD3976629309777F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{854EBA21-B016-4BC4-A18E-232C0D492BD6}"/>
   <bookViews>
     <workbookView showSheetTabs="0" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,368 +408,578 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A141"/>
+  <dimension ref="A1:B141"/>
   <sheetFormatPr defaultColWidth="12.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1">
         <v>168718.53390000001</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
+        <v>235975.2598</v>
+      </c>
+      <c r="B2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
         <v>293575.06390000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
+      <c r="B3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>196639.77559999999</v>
+      </c>
+      <c r="B4" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
         <v>195793.64920000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
+      <c r="B5" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>234627.0307</v>
+      </c>
+      <c r="B6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
         <v>292723.4558</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
+      <c r="B7" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>236707.74129999999</v>
+      </c>
+      <c r="B8" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
         <v>292996.16200000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1">
+      <c r="B9" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>294830.07299999997</v>
+      </c>
+      <c r="B10" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
         <v>294218.46299999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
+      <c r="B11" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1">
+        <v>195894.8082</v>
+      </c>
+      <c r="B12" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
         <v>196265.58009999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1">
+      <c r="B13" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1">
+        <v>106995.1059</v>
+      </c>
+      <c r="B14" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
         <v>167938.01010000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1">
+      <c r="B15" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>236033.37460000001</v>
+      </c>
+      <c r="B16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
         <v>234175.611</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1">
+      <c r="B17" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1">
+        <v>234363.17910000001</v>
+      </c>
+      <c r="B18" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
         <v>235345.10389999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1">
+      <c r="B19" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
+        <v>196207.71369999999</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="1">
         <v>146776.20790000001</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1">
+      <c r="B21" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1">
+        <v>294888.49959999998</v>
+      </c>
+      <c r="B22" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
         <v>166355.29990000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1">
+      <c r="B23" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
+        <v>296306.01380000002</v>
+      </c>
+      <c r="B24" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
         <v>195377.6636</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="1">
+      <c r="B25" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
+        <v>291625.94329999998</v>
+      </c>
+      <c r="B26" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
         <v>295583.6067</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1">
+      <c r="B27" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
+        <v>106673.9167</v>
+      </c>
+      <c r="B28" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
         <v>169020.56890000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1">
+      <c r="B29" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
+        <v>234675.65419999999</v>
+      </c>
+      <c r="B30" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
         <v>196442.1176</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1">
+      <c r="B31" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
+        <v>129414.12519999999</v>
+      </c>
+      <c r="B32" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
         <v>234953.29990000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1">
+      <c r="B33" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1">
+        <v>237259.17970000001</v>
+      </c>
+      <c r="B34" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
         <v>296284.47279999999</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1">
+      <c r="B35" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1">
+        <v>196500.21890000001</v>
+      </c>
+      <c r="B36" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
         <v>235508.4711</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1">
+      <c r="B37" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1">
+        <v>235100.58300000001</v>
+      </c>
+      <c r="B38" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="1">
         <v>235669.4883</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="1">
+      <c r="B39" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
+        <v>293519.20669999998</v>
+      </c>
+      <c r="B40" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
         <v>292738.65480000002</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="1">
+      <c r="B41" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="1">
+        <v>234383.24040000001</v>
+      </c>
+      <c r="B42" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="1">
         <v>105811.9371</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="1">
+      <c r="B43" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="1">
+        <v>91056.663159999996</v>
+      </c>
+      <c r="B44" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
         <v>117002.0159</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="1">
+      <c r="B45" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
+        <v>233223.18479999999</v>
+      </c>
+      <c r="B46" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="1">
         <v>147496.23689999999</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1">
+      <c r="B47" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="1">
+        <v>105289.799</v>
+      </c>
+      <c r="B48" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="1">
         <v>234249.55970000001</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1">
+      <c r="B49" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="1">
+        <v>236491.55069999999</v>
+      </c>
+      <c r="B50" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="1">
         <v>118031.8167</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="1">
+      <c r="B51" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="1">
+        <v>106518.9979</v>
+      </c>
+      <c r="B52" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="1">
         <v>233148.94399999999</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="1">
+      <c r="B53" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="1">
+        <v>393708.19380000001</v>
+      </c>
+      <c r="B54" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="1">
         <v>196194.33360000001</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="1">
+      <c r="B55" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="1">
+        <v>195061.63279999999</v>
+      </c>
+      <c r="B56" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
         <v>294668.18589999998</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="1">
+      <c r="B57" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
+        <v>234577.45509999999</v>
+      </c>
+      <c r="B58" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
         <v>234624.69649999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="1">
+      <c r="B59" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
+        <v>107817.58869999999</v>
+      </c>
+      <c r="B60" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
         <v>98728.991169999994</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="1">
+      <c r="B61" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
+        <v>233356.6384</v>
+      </c>
+      <c r="B62" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
         <v>234617.28899999999</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="1">
+      <c r="B63" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
+        <v>293651.9313</v>
+      </c>
+      <c r="B64" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
         <v>168684.01310000001</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="1">
+      <c r="B65" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
+        <v>196739.57639999999</v>
+      </c>
+      <c r="B66" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
         <v>106978.9179</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="1">
+      <c r="B67" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
+        <v>292826.84509999998</v>
+      </c>
+      <c r="B68" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
         <v>235517.4374</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="1">
-        <v>234421.9308</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="1">
-        <v>234910.7886</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="1">
-        <v>167062.4976</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="1">
-        <v>233538.73199999999</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="1">
-        <v>233009.85430000001</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="1">
-        <v>233291.38769999999</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="1">
-        <v>168440.32740000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="1">
-        <v>389687.10399999999</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="1">
-        <v>234912.3953</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="1">
-        <v>236016.13459999999</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="1">
-        <v>146109.5393</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="1">
-        <v>98484.26053</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="1">
-        <v>236623.2653</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="1">
-        <v>167828.99609999999</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="1">
-        <v>117335.14539999999</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="1">
-        <v>130673.8306</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="1">
-        <v>116925.977</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="1">
-        <v>196348.87849999999</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="1">
-        <v>115777.6122</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="1">
-        <v>392772.26630000002</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="1">
-        <v>235964.64230000001</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="1">
-        <v>167170.07870000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="1">
-        <v>233583.25279999999</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="1">
-        <v>234753.5019</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="1">
-        <v>117879.7135</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="1">
-        <v>237893.84229999999</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="1">
-        <v>130063.3029</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="1">
-        <v>394066.46970000002</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="1">
-        <v>293877.30070000002</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="1">
-        <v>391525.3493</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="1">
-        <v>235381.28450000001</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="1">
-        <v>168181.55350000001</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="1">
-        <v>193957.29389999999</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="1">
-        <v>294773.04739999998</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B69" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
-        <v>235254.37109999999</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="73" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="74" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="75" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="76" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="77" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="78" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="79" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="80" spans="1:1" ht="14.5" x14ac:dyDescent="0.35"/>
+        <v>168878.06049999999</v>
+      </c>
+      <c r="B70" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="73" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="74" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="75" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="76" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="77" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="78" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="79" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="80" spans="1:2" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="81" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="82" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="83" ht="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>